<commit_message>
used: pdf reader used
</commit_message>
<xml_diff>
--- a/Open-OMs.xlsx
+++ b/Open-OMs.xlsx
@@ -1,61 +1,37 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mao8ct\Desktop\PyAutomateSAP\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22B14257-0BA1-49C9-8745-8EE37AA3FAB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
-  <si>
-    <t>OM</t>
-  </si>
-  <si>
-    <t>Status</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="2">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -70,52 +46,93 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+  <cellXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -403,87 +420,385 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B12"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.42578125" bestFit="1" customWidth="1"/>
-  </cols>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B46"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="4">
-        <v>5197572</v>
-      </c>
-      <c r="B2" s="3"/>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="4">
-        <v>685601355769</v>
-      </c>
-      <c r="B3" s="3"/>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="4">
-        <v>685601364160</v>
-      </c>
-      <c r="B4" s="3"/>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="4">
-        <v>685601381667</v>
-      </c>
-      <c r="B5" s="3"/>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="4">
-        <v>685601355769</v>
-      </c>
-      <c r="B6" s="3"/>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="4">
-        <v>685601381337</v>
-      </c>
-      <c r="B7" s="3"/>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" s="4">
-        <v>685601381334</v>
-      </c>
-      <c r="B8" s="3"/>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" s="4">
-        <v>685601382736</v>
-      </c>
-      <c r="B9" s="3"/>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" s="4">
-        <v>685601382718</v>
-      </c>
-      <c r="B10" s="3"/>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" s="2">
-        <v>5198985</v>
-      </c>
-      <c r="B11" s="2"/>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" s="2">
-        <v>5199093</v>
-      </c>
-      <c r="B12" s="2"/>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>OM</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>5199787</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>5200014</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>5200306</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>5200305</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>5200138</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>5200106</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>5200160</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>5200226</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>5200179</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>5200112</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>5198091</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>5200744</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>5200452</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>685601401602</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>685601403471</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>685601403835</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>685601401311</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>685601397397</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>685601396692</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>685601397200</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>685601403832</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>685601400663</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>685601392573</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>685601400376</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>685601401209</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>685601382522</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>685601403583</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>685601385222</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>685601366315</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>685601392342</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>685601396398</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>685601396751</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>685601396752</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>685601381335</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>685601390226</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>355378</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>685601388256</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>685601400209</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>685601388256</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>685601389525</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>685601400329</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>685601400328</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>685601400327</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>685601400325</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>685601405585</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>